<commit_message>
Refresh executive summary: deployed smoke passes, art contracts supplied, website prototype
Update ten workstreams and website direction. Preserve executive inputs and prior qualifications on unchanged workstreams. Full gameplay acceptance, hardware performance, Master Control integration and launch readiness remain open.
</commit_message>
<xml_diff>
--- a/PKGameLabs-Executive-Workstreams.xlsx
+++ b/PKGameLabs-Executive-Workstreams.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workstreams" sheetId="1" r:id="Rf5cf6a795ba34336"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive direction" sheetId="2" r:id="R3c50611f09d448ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Authority and evidence" sheetId="3" r:id="R20dc18dfae064c0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workstreams" sheetId="1" r:id="R7d8adf807cfb4ca6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive direction" sheetId="2" r:id="R417cc4cd2e9b423a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Authority and evidence" sheetId="3" r:id="R41b63d9860ea42fd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -128,7 +128,7 @@
         <x:color rgb="FF9D3029"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE5E2"/>
         </x:patternFill>
       </x:fill>
@@ -139,7 +139,7 @@
         <x:color rgb="FF805B15"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0D9"/>
         </x:patternFill>
       </x:fill>
@@ -150,7 +150,7 @@
         <x:color rgb="FF6A3983"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF4E8FA"/>
         </x:patternFill>
       </x:fill>
@@ -161,7 +161,7 @@
         <x:color rgb="FF5A6574"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE9EDF2"/>
         </x:patternFill>
       </x:fill>
@@ -435,7 +435,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="3" t="str">
-        <x:v>Reviewed October 5, 2026 (EDT). Status is delivery health, not a personnel rating.</x:v>
+        <x:v>Reviewed October 5, 2026, 03:49 EDT intake. Unchanged rows retain prior evidence. Status describes delivery health.</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -479,13 +479,13 @@
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="C6" s="11" t="str">
-        <x:v>Executive decisions adopted; C-Suite becomes the single executive reporting home. Website remains the primary delivery obligation.</x:v>
+        <x:v>Website prototype now reported with working player-reference features and PKQuest art. C-Suite reporting is published.</x:v>
       </x:c>
       <x:c r="D6" s="11" t="str">
-        <x:v>Produce a concrete website handoff; reconcile authority and conflicting workstream reports.</x:v>
+        <x:v>Close website brand direction and launch scope with Marketing. Prioritize interactive Windows acceptance.</x:v>
       </x:c>
       <x:c r="E6" s="11" t="str">
-        <x:v>No new approval needed. Website delivery is mine to close.</x:v>
+        <x:v>Help secure a hardware Windows playtest and keep launch scope bounded.</x:v>
       </x:c>
       <x:c r="F6" s="12" t="str"/>
     </x:row>
@@ -515,13 +515,13 @@
         <x:v>At risk</x:v>
       </x:c>
       <x:c r="C8" s="11" t="str">
-        <x:v>Integrated Windows candidate built and exact test pair verified. R29 remains governing; deployed game has not advanced with that candidate.</x:v>
+        <x:v>Integrated game deployed with matched PKTest 0.7.3. Windows New Game, radar and control-bridge smoke pass. Full acceptance remains open.</x:v>
       </x:c>
       <x:c r="D8" s="11" t="str">
-        <x:v>Finish runtime bindings, deploy matching bytes, obtain fresh Windows gameplay/visual/performance evidence.</x:v>
+        <x:v>Complete interactive gameplay, visual and hardware-performance evidence on the exact deployed pair. Finish remaining runtime bindings.</x:v>
       </x:c>
       <x:c r="E8" s="11" t="str">
-        <x:v>Highest leverage: ensure the authorized Windows execution lane has an available operator and machine.</x:v>
+        <x:v>Highest leverage: arrange a hardware Windows playtest with an accountable operator.</x:v>
       </x:c>
       <x:c r="F8" s="12" t="str"/>
     </x:row>
@@ -533,13 +533,13 @@
         <x:v>Dependent</x:v>
       </x:c>
       <x:c r="C9" s="6" t="str">
-        <x:v>Recovered New Player producer semantics are integrated in a new Windows candidate; contract checks pass. This is not gameplay acceptance.</x:v>
+        <x:v>A189 numeric rendering is merged and Windows build/contracts pass. Deployed smoke-tested game still uses the earlier source.</x:v>
       </x:c>
       <x:c r="D9" s="6" t="str">
-        <x:v>Close new producer/consumer identity and custody evidence; consume fresh W01–W18 results. Oblivion schema work remains a separate dependency.</x:v>
+        <x:v>Validate A189 in its own deployed candidate. Integrate Oblivion Core semantics and required acceptance fixtures.</x:v>
       </x:c>
       <x:c r="E9" s="6" t="str">
-        <x:v>No new design decision evidenced. Keep acceptance tied to the exact new pair.</x:v>
+        <x:v>No new design decision evidenced. Source completion does not establish deployed acceptance.</x:v>
       </x:c>
       <x:c r="F9" s="12" t="str"/>
     </x:row>
@@ -551,13 +551,13 @@
         <x:v>Dependent</x:v>
       </x:c>
       <x:c r="C10" s="11" t="str">
-        <x:v>Acceptance tooling is prepared. PKStudio now lists PKTest 0.7.1; the inspected integrated game lock uses 0.7.0.</x:v>
+        <x:v>PKTest 0.7.3 runtime repair deployed. Matched Windows smoke passes New Game, radar and control bridge; 9 native regressions pass.</x:v>
       </x:c>
       <x:c r="D10" s="11" t="str">
-        <x:v>Run W01–W18 on the exact locked Windows pair. Using 0.7.1 requires a fresh lock and fresh evidence.</x:v>
+        <x:v>Complete W01–W18 and hardware visual/performance acceptance. Historical 0.7.0 locks remain historical.</x:v>
       </x:c>
       <x:c r="E10" s="11" t="str">
-        <x:v>Existing Windows-lane authorization stands; help with execution access only if still unavailable.</x:v>
+        <x:v>Windows automation access is demonstrated. Help with interactive hardware testing rather than a generic lane procurement.</x:v>
       </x:c>
       <x:c r="F10" s="12" t="str"/>
     </x:row>
@@ -584,16 +584,16 @@
         <x:v>Art Director</x:v>
       </x:c>
       <x:c r="B12" s="11" t="str">
-        <x:v>Reconcile</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="C12" s="11" t="str">
-        <x:v>Spawn-100 art closed at 11,047 approved placements; named NPC models ready. Full production-art approval authority is active.</x:v>
+        <x:v>Creature-lane conflict reconciled: directional coverage is active; five separate boss packages remain contract-gated. Art approval queue is growing.</x:v>
       </x:c>
       <x:c r="D12" s="11" t="str">
-        <x:v>Resolve differing Wave-1 lane reports: Director reports production can proceed; PKArt still reports missing contracts.</x:v>
+        <x:v>Review exact creature bindings and Bone/Keeper candidates. Resolve website branding request and remaining boss contracts.</x:v>
       </x:c>
       <x:c r="E12" s="11" t="str">
-        <x:v>No second Executive art gate. Chief Integrator reconciles scope and receipt identity.</x:v>
+        <x:v>No second Executive art gate. Protect Art Director review capacity and prioritize the queue.</x:v>
       </x:c>
       <x:c r="F12" s="12" t="str"/>
     </x:row>
@@ -605,13 +605,13 @@
         <x:v>Dependent</x:v>
       </x:c>
       <x:c r="C13" s="6" t="str">
-        <x:v>Spawn-100 final art package is approved; grass family is closed. Wave-1 preflight identifies missing IDs, profiles and consumer bindings.</x:v>
+        <x:v>Zone-1 batch registers 15 creatures and 120 static directional/corpse frames for review. Oblivion profiles and Lantern door consumer now supplied.</x:v>
       </x:c>
       <x:c r="D13" s="6" t="str">
-        <x:v>Match each production lane to Content/Wiring contracts and current Art Director order; then return discrete approved families.</x:v>
+        <x:v>Consume new contracts, obtain Art Director dispositions and export exact runtime assets. UI effects still need accepted stable IDs.</x:v>
       </x:c>
       <x:c r="E13" s="6" t="str">
-        <x:v>No blanket pixel-production approval needed. Escalate only a concrete authority conflict.</x:v>
+        <x:v>Help enforce handoff closure. Review boards and binding metadata are not approved runtime deliveries.</x:v>
       </x:c>
       <x:c r="F13" s="12" t="str"/>
     </x:row>
@@ -623,13 +623,13 @@
         <x:v>Dependent</x:v>
       </x:c>
       <x:c r="C14" s="11" t="str">
-        <x:v>Art–Content interface v2 defines stable semantics and one Oblivion family: 11 wearables plus 2 separate tools.</x:v>
+        <x:v>Oblivion Core expands the unified family to 12 wearables plus 2 tools. Adaptive behavior contract and 25 acceptance fixtures are specified.</x:v>
       </x:c>
       <x:c r="D14" s="11" t="str">
-        <x:v>Resolve exact boss/item/profile contracts and authored Story Spot/location inputs; coordinate spatial anchors with Map/Wiring.</x:v>
+        <x:v>Build/Wiring must implement and validate Core identity, adaptation, atomic equipment changes and persistence.</x:v>
       </x:c>
       <x:c r="E14" s="11" t="str">
-        <x:v>No unresolved Executive design choice verified; current requests are specialist handoffs.</x:v>
+        <x:v>No new Executive choice evidenced. Preserve one item identity across adaptation and trade.</x:v>
       </x:c>
       <x:c r="F14" s="12" t="str"/>
     </x:row>
@@ -641,13 +641,13 @@
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="C15" s="6" t="str">
-        <x:v>Specialist deliveries now include Phase75 dialogue parity, Phase76 shared Hideouts and Phase77 location recovery. Publication is not adoption.</x:v>
+        <x:v>Published 13 Oblivion presentation profiles plus existing Core profile, and the open/closed Lantern door contract for four consumers.</x:v>
       </x:c>
       <x:c r="D15" s="6" t="str">
-        <x:v>Integrate the current specialist changes and reconcile PKArt bindings; preserve identities and saved state.</x:v>
+        <x:v>PKArt must consume these contracts; Build Master must integrate matching art and runtime bindings.</x:v>
       </x:c>
       <x:c r="E15" s="6" t="str">
-        <x:v>None identified. Keep adoption responsibility with Build Master.</x:v>
+        <x:v>None identified. Previously missing contracts now need acknowledged adoption.</x:v>
       </x:c>
       <x:c r="F15" s="12" t="str"/>
     </x:row>
@@ -695,13 +695,13 @@
         <x:v>Dependent</x:v>
       </x:c>
       <x:c r="C18" s="11" t="str">
-        <x:v>Content and Art Studio 0.6.3 are listed as runnable; PKTest 0.7.1 is listed. Native selected-target identity checks passed on Windows.</x:v>
+        <x:v>Content and Art Studio 0.6.3 remain listed; PKTest is now 0.7.3. Runtime repair explicitly does not embed PKTest in Master Control.</x:v>
       </x:c>
       <x:c r="D18" s="11" t="str">
-        <x:v>Deliver Master Control host, target previews, validators and certified atomic LIVE LOCAL publishing.</x:v>
+        <x:v>Deliver integrated Master Control TEST and certify atomic LIVE LOCAL publishing. Studio currently writes drafts only.</x:v>
       </x:c>
       <x:c r="E18" s="11" t="str">
-        <x:v>No new approval evidenced. Packaging success does not close publisher certification.</x:v>
+        <x:v>Keep runtime packaging, suite integration and publisher certification as separate closure checks.</x:v>
       </x:c>
       <x:c r="F18" s="12" t="str"/>
     </x:row>
@@ -731,13 +731,13 @@
         <x:v>At risk</x:v>
       </x:c>
       <x:c r="C20" s="11" t="str">
-        <x:v>Department reports Strategy, Copy, PR and launch controls ready; Creative remains dependent on captures. Five named lead appointments are not verified.</x:v>
+        <x:v>Website prototype reports working search, reference viewer and preparation tools using PKQuest art. Website-specific branding approval is pending.</x:v>
       </x:c>
       <x:c r="D20" s="11" t="str">
-        <x:v>Hand off website content and approved Windows visuals; verify destinations and named functional ownership.</x:v>
+        <x:v>Obtain Art Director brand direction and a scoped launch roadmap. Account, download, raffle and community services are not live.</x:v>
       </x:c>
       <x:c r="E20" s="11" t="str">
-        <x:v>Reconcile existing appointments before procuring duplicates. Activate any truly vacant Strategy/Copy seats first.</x:v>
+        <x:v>Prioritize real player services and PKQuest branding. Named lead appointments remain unverified.</x:v>
       </x:c>
       <x:c r="F20" s="12" t="str"/>
     </x:row>
@@ -791,7 +791,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4cf10ad7d52f4a23"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re383c153474840eb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -943,10 +943,10 @@
         <x:v>Website</x:v>
       </x:c>
       <x:c r="C12" s="11" t="str">
-        <x:v>Tibia-inspired experience; no external ads. Chief Integrator accountable; Marketing supplies content and launch preparation.</x:v>
+        <x:v>Use Tibia as a functional reference for player services and navigation. Use PKQuest art and Art Director branding. No external ads. Chief Integrator accountable.</x:v>
       </x:c>
       <x:c r="D12" s="11" t="str">
-        <x:v>Executive decision intake</x:v>
+        <x:v>Executive correction recorded in Marketing branding check-in, October 5, 2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="48" customHeight="1">
@@ -1022,7 +1022,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc572e7e72b4f451a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b8511b64af14394"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1056,7 +1056,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="3" t="str">
-        <x:v>Sources reviewed October 5, 2026. Reported updates and unresolved conflicts are explicitly qualified.</x:v>
+        <x:v>October 5, 2026, 03:49 EDT intake. New primary evidence replaces affected rows; other rows retain earlier qualifications.</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -1095,13 +1095,13 @@
         <x:v>Reports to Executive; PK Game Labs scope; continuity and succession owner.</x:v>
       </x:c>
       <x:c r="C6" s="11" t="str">
-        <x:v>Direct Executive instructions in this conversation, 2026-10-05.</x:v>
+        <x:v>Marketing–Art Director branding check-in, 2026-10-05 (07:31Z); C-Suite main e1d4785.</x:v>
       </x:c>
       <x:c r="D6" s="11" t="str">
-        <x:v>Direct instruction</x:v>
+        <x:v>Primary producer report + verified repo</x:v>
       </x:c>
       <x:c r="E6" s="11" t="str">
-        <x:v>Website accountability retained; no team interruption or appointment invented.</x:v>
+        <x:v>Website functionality is producer-reported, not independently exercised in this refresh.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="64" customHeight="1">
@@ -1129,13 +1129,13 @@
         <x:v>Technical integration, packed runtime, build/release acceptance. New Build Master succession remains governing.</x:v>
       </x:c>
       <x:c r="C8" s="11" t="str">
-        <x:v>https://github.com/houdinicap/PKGameLabs/blob/f8db5ea9531872a26f6b528d51c85d8d432d9076/WORKSTREAM-CHECKPOINT.md</x:v>
+        <x:v>PKGameLabs-BuildMaster-Status.json v69, pkTestRuntimeRepair; GitHub run 37271845473; checkpoint d6b017243be387ccab1bd1c57275bc97fd1a26c5.</x:v>
       </x:c>
       <x:c r="D8" s="11" t="str">
-        <x:v>Primary Git checkpoint</x:v>
+        <x:v>Primary Build Master record</x:v>
       </x:c>
       <x:c r="E8" s="11" t="str">
-        <x:v>Newer appended integration evidence supersedes stale v68 coordination-summary blockers. Historical A159 archive absence is not the blocker for the new integrated pair.</x:v>
+        <x:v>Game f3752788… / PKTest 952928a6… matched. Hosted Windows Mesa llvmpipe smoke is not hardware performance or full acceptance.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="64" customHeight="1">
@@ -1146,13 +1146,13 @@
         <x:v>Gameplay/state contracts; Build Master owns adopted source and binaries.</x:v>
       </x:c>
       <x:c r="C9" s="6" t="str">
-        <x:v>https://github.com/houdinicap/PKGameLabs/blob/f8db5ea9531872a26f6b528d51c85d8d432d9076/WORKSTREAM-CHECKPOINT.md; latest AI conversation return retrieved 2026-10-05.</x:v>
+        <x:v>PKQuest-AI-Framework-R29-A189-Implementation-Receipt-2026-10-05.md; Build Master v69 runtime repair.</x:v>
       </x:c>
       <x:c r="D9" s="6" t="str">
-        <x:v>Primary + reported update</x:v>
+        <x:v>Primary specialist + integrator records</x:v>
       </x:c>
       <x:c r="E9" s="6" t="str">
-        <x:v>Integrated candidate identity differs from original A159/A159R. No inherited Windows acceptance.</x:v>
+        <x:v>51 renderer/edge checks, 38 topology checks, 22 recipe checks reported passing. A189 is not the deployed smoke-tested binary.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="64" customHeight="1">
@@ -1163,13 +1163,13 @@
         <x:v>Test tooling and evidence; no self-certification of an unexecuted game.</x:v>
       </x:c>
       <x:c r="C10" s="11" t="str">
-        <x:v>https://github.com/houdinicap/PKGameLabs/blob/f8db5ea9531872a26f6b528d51c85d8d432d9076/WORKSTREAM-CHECKPOINT.md; https://github.com/houdinicap/PKStudio/blob/main/README.md</x:v>
+        <x:v>Build Master v69 pkTestRuntimeRepair; https://github.com/houdinicap/PKStudio/blob/main/README.md</x:v>
       </x:c>
       <x:c r="D10" s="11" t="str">
-        <x:v>Primary Git files</x:v>
+        <x:v>Primary integrator + repository</x:v>
       </x:c>
       <x:c r="E10" s="11" t="str">
-        <x:v>PKTest 0.7.1 availability does not alter the inspected 0.7.0 game lock.</x:v>
+        <x:v>0.7.3-runtime-repair is a new matched pair. Smoke passes; fullAcceptance=false. Historical 0.7.0 locks unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="64" customHeight="1">
@@ -1197,13 +1197,13 @@
         <x:v>Executive-delegated full artistic direction and production-art approval.</x:v>
       </x:c>
       <x:c r="C12" s="11" t="str">
-        <x:v>PKQ-AD-R29-READY-016; PKQ-AD-R29-COVERAGE-015; latest Art Director return retrieved 2026-10-05.</x:v>
+        <x:v>PKArt ACTIVE-CREATURE-LANE-REVIEW-v1; ZONE1-CREATURE-BINDING-BATCH-v1-REVIEW; BONE-KEEPER-ART-DIRECTOR-REVIEW-INTAKE-v1; Marketing branding check-in (all 2026-10-05).</x:v>
       </x:c>
       <x:c r="D12" s="11" t="str">
-        <x:v>Primary + reported update</x:v>
+        <x:v>Primary producer handoffs</x:v>
       </x:c>
       <x:c r="E12" s="11" t="str">
-        <x:v>Later Director report names a different production order; reconcile by exact lane rather than assuming PKArt is cleared.</x:v>
+        <x:v>Directional lane and five COVERAGE-015 boss packages are distinct. Pending reviews do not imply approval.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="64" customHeight="1">
@@ -1214,13 +1214,13 @@
         <x:v>Production assets under Art Director; no gameplay identity/footprint authority.</x:v>
       </x:c>
       <x:c r="C13" s="6" t="str">
-        <x:v>PKQuest-PKArt-R29-WAVE1-UNBLOCK-REQUEST.json; Oblivion delta review; PKQ-AD-R29-READY-016.</x:v>
+        <x:v>PKArt Zone1 creature batch review v1; ContentWiring Oblivion profiles v1 and Lantern door consumer v1; UI &amp; Effects Combat Effect Preflight v1 (2026-10-05).</x:v>
       </x:c>
       <x:c r="D13" s="6" t="str">
-        <x:v>Primary files + later report</x:v>
+        <x:v>Primary producer contracts</x:v>
       </x:c>
       <x:c r="E13" s="6" t="str">
-        <x:v>Content interface v2 has logical Oblivion targets; PKArt still requests exact per-definition profile reconciliation. This is an intake conflict, not proven global absence.</x:v>
+        <x:v>15 creatures / 120 frames are binding metadata awaiting Art Director review. Armor-stop and resisted-magic labels are not accepted runtime IDs.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="64" customHeight="1">
@@ -1231,13 +1231,13 @@
         <x:v>Semantic IDs, gameplay identities, logical presentation contracts; Map owns coordinates.</x:v>
       </x:c>
       <x:c r="C14" s="11" t="str">
-        <x:v>PKQuest-Art-Content-Interface-Manifest-v2.txt; Warehouse Checkpoint07; PKArt Wave1 request.</x:v>
+        <x:v>PKQuest-Oblivion-Core-Integration-Handoff-v1.txt, Content Pack150, 2026-10-05.</x:v>
       </x:c>
       <x:c r="D14" s="11" t="str">
-        <x:v>Primary files</x:v>
+        <x:v>Primary semantic contract</x:v>
       </x:c>
       <x:c r="E14" s="11" t="str">
-        <x:v>11 wearable Oblivion definitions; Shovel/Pickaxe excluded from wearable set membership.</x:v>
+        <x:v>12 wearable definitions including Core, plus 2 nonwearable tools. 25 fixtures are required, not reported executed.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="64" customHeight="1">
@@ -1248,13 +1248,13 @@
         <x:v>Runtime contract wiring and specialist implementations; Build Master integrates.</x:v>
       </x:c>
       <x:c r="C15" s="6" t="str">
-        <x:v>Library inventory: Phase75 (05:26Z), Phase76 (05:36Z), Phase77 (05:49Z), 2026-10-05; Warehouse Checkpoint07.</x:v>
+        <x:v>PKQuest-ContentWiring-R29-OBLIVION-PRESENTATION-PROFILES-v1-2026-10-05.json; PKQuest-ContentWiring-R29-LANTERN-DOOR-OPEN-CONSUMER-v1-2026-10-05.json.</x:v>
       </x:c>
       <x:c r="D15" s="6" t="str">
-        <x:v>Package existence + primary context</x:v>
+        <x:v>Primary contract files</x:v>
       </x:c>
       <x:c r="E15" s="6" t="str">
-        <x:v>Latest ZIP bodies not audited in this intake; no tests or runtime adoption inferred from filenames.</x:v>
+        <x:v>13 newly resolved profiles plus Core. Four door consumers share one open state family. No art approval or integration acceptance claimed.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="64" customHeight="1">
@@ -1299,13 +1299,13 @@
         <x:v>Studio tools; Build Master target services and integration; LIVE LOCAL certification boundary remains.</x:v>
       </x:c>
       <x:c r="C18" s="11" t="str">
-        <x:v>https://github.com/houdinicap/PKStudio/blob/main/README.md; https://github.com/houdinicap/PKGameLabs/blob/f8db5ea9531872a26f6b528d51c85d8d432d9076/WORKSTREAM-CHECKPOINT.md</x:v>
+        <x:v>https://github.com/houdinicap/PKStudio/blob/main/README.md (PKTest0.7.3); Build Master v69 pkTestRuntimeRepair.</x:v>
       </x:c>
       <x:c r="D18" s="11" t="str">
-        <x:v>Primary Git files</x:v>
+        <x:v>Primary repository + integrator</x:v>
       </x:c>
       <x:c r="E18" s="11" t="str">
-        <x:v>0.6.4 was reported as an unsaved attempt; do not present it as deployed.</x:v>
+        <x:v>masterControlEmbedding=false. Studio draft writing does not enable authoritative promotion.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="64" customHeight="1">
@@ -1333,13 +1333,13 @@
         <x:v>VP owns Marketing; functional leaders within department; Chronicle independent.</x:v>
       </x:c>
       <x:c r="C20" s="11" t="str">
-        <x:v>Marketing Chief Integrator check-in; procurement manifest; Snapshot2; latest Marketing Department conversation return.</x:v>
+        <x:v>PKQuest-Marketing-ArtDirector-Branding-Checkin-2026-10-05.txt (07:31Z).</x:v>
       </x:c>
       <x:c r="D20" s="11" t="str">
-        <x:v>Primary files + reported update</x:v>
+        <x:v>Primary Marketing report</x:v>
       </x:c>
       <x:c r="E20" s="11" t="str">
-        <x:v>Active department reported; individual named seat appointments still need reconciliation. No duplicate staffing demand.</x:v>
+        <x:v>Working features are reported, not independently tested. Brand request receipt/reply unconfirmed. Public launch services remain incomplete.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="64" customHeight="1">
@@ -1379,7 +1379,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd1a6fafc56ee43ad"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8611854dd1141ac"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>